<commit_message>
#31 eSpark BOM 20,50,100,500 and 1000 Quantity Added
</commit_message>
<xml_diff>
--- a/Design Files/LoRaWAN-Module-v2.0/BOM/eSpark_BOM_LoRaWAN-Module-v2.0.xlsx
+++ b/Design Files/LoRaWAN-Module-v2.0/BOM/eSpark_BOM_LoRaWAN-Module-v2.0.xlsx
@@ -13,13 +13,18 @@
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="20 Boards" sheetId="2" r:id="rId2"/>
+    <sheet name="50 Boards" sheetId="3" r:id="rId3"/>
+    <sheet name="100 Boards" sheetId="4" r:id="rId4"/>
+    <sheet name="500 Boards" sheetId="5" r:id="rId5"/>
+    <sheet name="1000 Boards" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="92">
   <si>
     <t>Component list</t>
   </si>
@@ -235,6 +240,66 @@
   </si>
   <si>
     <t>C1509213</t>
+  </si>
+  <si>
+    <t>Quantity (20 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (20 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (20 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (20 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (50 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (50 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (50 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (50 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (100 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (100 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (500 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (500 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (500 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (500 Boards)</t>
+  </si>
+  <si>
+    <t>Quantity (1000 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (1000 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (1000 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (1000 Boards)</t>
   </si>
 </sst>
 </file>
@@ -706,7 +771,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -879,6 +944,15 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -910,6 +984,50 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -977,6 +1095,276 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="29927550" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19230975" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19230975" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19230975" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19230975" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19230975" y="620017"/>
           <a:ext cx="1714500" cy="1104008"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1287,15 +1675,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="65"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1345,7 +1733,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="66"/>
+      <c r="S3" s="69"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1370,7 +1758,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="67"/>
+      <c r="S4" s="70"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1395,7 +1783,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="67"/>
+      <c r="S5" s="70"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1416,7 +1804,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="67"/>
+      <c r="S6" s="70"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1437,7 +1825,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="67"/>
+      <c r="S7" s="70"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1458,7 +1846,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="67"/>
+      <c r="S8" s="70"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1724,12 +2112,18 @@
         <f t="shared" ref="M13" si="3">L13*5</f>
         <v>5</v>
       </c>
-      <c r="N13" s="51"/>
-      <c r="O13" s="63"/>
-      <c r="P13" s="52"/>
+      <c r="N13" s="51">
+        <v>6</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.81620000000000004</v>
+      </c>
       <c r="Q13" s="52">
         <f t="shared" ref="Q13" si="4">P13*N13</f>
-        <v>0</v>
+        <v>4.8971999999999998</v>
       </c>
       <c r="R13" s="51"/>
       <c r="S13" s="59"/>
@@ -1846,61 +2240,61 @@
       <c r="R15" s="51"/>
       <c r="S15" s="39"/>
     </row>
-    <row r="16" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="47">
+    <row r="16" spans="1:19" s="85" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="77"/>
+      <c r="B16" s="86">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="79" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="51" t="s">
+      <c r="D16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="G16" s="51" t="s">
+      <c r="F16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="81" t="s">
         <v>65</v>
       </c>
-      <c r="H16" s="51" t="s">
+      <c r="H16" s="81" t="s">
         <v>66</v>
       </c>
-      <c r="I16" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="J16" s="51" t="s">
+      <c r="I16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="81" t="s">
         <v>67</v>
       </c>
-      <c r="K16" s="51" t="s">
-        <v>53</v>
-      </c>
-      <c r="L16" s="51">
+      <c r="K16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="81">
         <v>1</v>
       </c>
-      <c r="M16" s="51">
+      <c r="M16" s="81">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="N16" s="51">
+      <c r="N16" s="81">
         <v>5</v>
       </c>
-      <c r="O16" s="60" t="s">
+      <c r="O16" s="82" t="s">
         <v>52</v>
       </c>
-      <c r="P16" s="52">
+      <c r="P16" s="83">
         <v>1.0126999999999999</v>
       </c>
-      <c r="Q16" s="52">
+      <c r="Q16" s="83">
         <f t="shared" si="6"/>
         <v>5.0634999999999994</v>
       </c>
-      <c r="R16" s="51"/>
-      <c r="S16" s="39"/>
+      <c r="R16" s="81"/>
+      <c r="S16" s="92"/>
     </row>
     <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -1916,17 +2310,17 @@
       <c r="K17" s="45"/>
       <c r="L17" s="45"/>
       <c r="M17" s="45"/>
-      <c r="N17" s="72" t="s">
+      <c r="N17" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="O17" s="73"/>
-      <c r="P17" s="73"/>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
       <c r="Q17" s="48">
         <f>SUM(Q10:Q16)</f>
-        <v>31.381500000000003</v>
-      </c>
-      <c r="R17" s="68"/>
-      <c r="S17" s="69"/>
+        <v>36.278700000000001</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
     </row>
     <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -1942,17 +2336,17 @@
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
-      <c r="N18" s="72" t="s">
+      <c r="N18" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="O18" s="73"/>
-      <c r="P18" s="73"/>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
       <c r="Q18" s="49">
         <f>Q17/5</f>
-        <v>6.2763000000000009</v>
-      </c>
-      <c r="R18" s="70"/>
-      <c r="S18" s="71"/>
+        <v>7.2557400000000003</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1968,9 +2362,3659 @@
     <hyperlink ref="O15" r:id="rId3"/>
     <hyperlink ref="O14" r:id="rId4"/>
     <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="69"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="70"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="70"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="70"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="70"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="70"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="64"/>
+      <c r="B10" s="46">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="37">
+        <v>1</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*20</f>
+        <v>20</v>
+      </c>
+      <c r="N10" s="51">
+        <v>100</v>
+      </c>
+      <c r="O10" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" s="52">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="Q10" s="38">
+        <f>P10*N10</f>
+        <v>0.52</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="65"/>
+    </row>
+    <row r="11" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="64"/>
+      <c r="B11" s="47">
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="51" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="51">
+        <v>1</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M16" si="1">L11*20</f>
+        <v>20</v>
+      </c>
+      <c r="N11" s="51">
+        <v>100</v>
+      </c>
+      <c r="O11" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="52">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q11" s="52">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>0.24</v>
+      </c>
+      <c r="R11" s="51"/>
+      <c r="S11" s="51"/>
+    </row>
+    <row r="12" spans="1:19" s="66" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="64"/>
+      <c r="B12" s="46">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="61">
+        <v>1</v>
+      </c>
+      <c r="M12" s="61">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" s="61"/>
+      <c r="S12" s="59"/>
+    </row>
+    <row r="13" spans="1:19" s="66" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="47">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="K13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="51">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N13" s="51">
+        <v>21</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.66659999999999997</v>
+      </c>
+      <c r="Q13" s="52">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>13.9986</v>
+      </c>
+      <c r="R13" s="51"/>
+      <c r="S13" s="59"/>
+    </row>
+    <row r="14" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="64"/>
+      <c r="B14" s="46">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="37">
+        <v>2</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="N14" s="37">
+        <v>100</v>
+      </c>
+      <c r="O14" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="38">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q14" s="38">
+        <f>P14*N14</f>
+        <v>0.13</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="59"/>
+    </row>
+    <row r="15" spans="1:19" s="66" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="64"/>
+      <c r="B15" s="47">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="51">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N15" s="51">
+        <v>21</v>
+      </c>
+      <c r="O15" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="52">
+        <v>4.4610000000000003</v>
+      </c>
+      <c r="Q15" s="52">
+        <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
+        <v>93.681000000000012</v>
+      </c>
+      <c r="R15" s="51"/>
+      <c r="S15" s="39"/>
+    </row>
+    <row r="16" spans="1:19" s="66" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="64"/>
+      <c r="B16" s="47">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="51">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N16" s="51">
+        <v>20</v>
+      </c>
+      <c r="O16" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="52">
+        <v>0.85399999999999998</v>
+      </c>
+      <c r="Q16" s="52">
+        <f t="shared" si="4"/>
+        <v>17.079999999999998</v>
+      </c>
+      <c r="R16" s="51"/>
+      <c r="S16" s="39"/>
+    </row>
+    <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="48">
+        <f>SUM(Q10:Q16)</f>
+        <v>125.64960000000001</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
+    </row>
+    <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="49">
+        <f>Q17/20</f>
+        <v>6.2824800000000005</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="R17:S18"/>
+    <mergeCell ref="N18:P18"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O15" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="69"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="70"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="70"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="70"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="70"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="70"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="64"/>
+      <c r="B10" s="46">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="37">
+        <v>1</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*50</f>
+        <v>50</v>
+      </c>
+      <c r="N10" s="51">
+        <v>100</v>
+      </c>
+      <c r="O10" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" s="52">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="Q10" s="38">
+        <f>P10*N10</f>
+        <v>0.52</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="65"/>
+    </row>
+    <row r="11" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="64"/>
+      <c r="B11" s="47">
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="51" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="51">
+        <v>1</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M16" si="1">L11*50</f>
+        <v>50</v>
+      </c>
+      <c r="N11" s="51">
+        <v>100</v>
+      </c>
+      <c r="O11" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="52">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q11" s="52">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>0.24</v>
+      </c>
+      <c r="R11" s="51"/>
+      <c r="S11" s="51"/>
+    </row>
+    <row r="12" spans="1:19" s="66" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="64"/>
+      <c r="B12" s="46">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="61">
+        <v>1</v>
+      </c>
+      <c r="M12" s="61">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="N12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" s="61"/>
+      <c r="S12" s="59"/>
+    </row>
+    <row r="13" spans="1:19" s="66" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="47">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="K13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="51">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="N13" s="51">
+        <v>51</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.59189999999999998</v>
+      </c>
+      <c r="Q13" s="52">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>30.186899999999998</v>
+      </c>
+      <c r="R13" s="51"/>
+      <c r="S13" s="59"/>
+    </row>
+    <row r="14" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="64"/>
+      <c r="B14" s="46">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="37">
+        <v>2</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N14" s="37">
+        <v>200</v>
+      </c>
+      <c r="O14" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="38">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q14" s="38">
+        <f>P14*N14</f>
+        <v>0.26</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="59"/>
+    </row>
+    <row r="15" spans="1:19" s="66" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="64"/>
+      <c r="B15" s="47">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="51">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="N15" s="51">
+        <v>51</v>
+      </c>
+      <c r="O15" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="52">
+        <v>4.3240999999999996</v>
+      </c>
+      <c r="Q15" s="52">
+        <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
+        <v>220.52909999999997</v>
+      </c>
+      <c r="R15" s="51"/>
+      <c r="S15" s="39"/>
+    </row>
+    <row r="16" spans="1:19" s="66" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="64"/>
+      <c r="B16" s="47">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="51">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="N16" s="51">
+        <v>50</v>
+      </c>
+      <c r="O16" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="52">
+        <v>0.76780000000000004</v>
+      </c>
+      <c r="Q16" s="52">
+        <f t="shared" si="4"/>
+        <v>38.39</v>
+      </c>
+      <c r="R16" s="51"/>
+      <c r="S16" s="39"/>
+    </row>
+    <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="48">
+        <f>SUM(Q10:Q16)</f>
+        <v>290.12599999999998</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
+    </row>
+    <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="49">
+        <f>Q17/50</f>
+        <v>5.8025199999999995</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="R17:S18"/>
+    <mergeCell ref="N18:P18"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O15" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="69"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="70"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="70"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="70"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="70"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="70"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="77"/>
+      <c r="B10" s="78">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="80" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="80" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="80" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="80" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="80" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="80">
+        <v>1</v>
+      </c>
+      <c r="M10" s="80">
+        <f>L10*100</f>
+        <v>100</v>
+      </c>
+      <c r="N10" s="81">
+        <v>200</v>
+      </c>
+      <c r="O10" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" s="83">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="Q10" s="84">
+        <f>P10*N10</f>
+        <v>1.04</v>
+      </c>
+      <c r="R10" s="80"/>
+      <c r="S10" s="50"/>
+    </row>
+    <row r="11" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="77"/>
+      <c r="B11" s="86">
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="81" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="81" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="81" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="87" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="81" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="81" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="81" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="81">
+        <v>1</v>
+      </c>
+      <c r="M11" s="80">
+        <f t="shared" ref="M11:M16" si="1">L11*100</f>
+        <v>100</v>
+      </c>
+      <c r="N11" s="81">
+        <v>200</v>
+      </c>
+      <c r="O11" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="83">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q11" s="83">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>0.48</v>
+      </c>
+      <c r="R11" s="81"/>
+      <c r="S11" s="81"/>
+    </row>
+    <row r="12" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="77"/>
+      <c r="B12" s="78">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="87" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="87" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="87" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="87">
+        <v>1</v>
+      </c>
+      <c r="M12" s="87">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" s="89" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" s="89" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" s="87"/>
+      <c r="S12" s="90"/>
+    </row>
+    <row r="13" spans="1:19" s="85" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A13" s="77"/>
+      <c r="B13" s="86">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="79" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="81" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="81" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="81" t="s">
+        <v>71</v>
+      </c>
+      <c r="K13" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="81">
+        <v>1</v>
+      </c>
+      <c r="M13" s="80">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N13" s="81">
+        <v>101</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.51870000000000005</v>
+      </c>
+      <c r="Q13" s="83">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>52.388700000000007</v>
+      </c>
+      <c r="R13" s="81"/>
+      <c r="S13" s="90"/>
+    </row>
+    <row r="14" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="77"/>
+      <c r="B14" s="78">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="88" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="80" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="80" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="80" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="80" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="80" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="80" t="s">
+        <v>61</v>
+      </c>
+      <c r="K14" s="80" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="80">
+        <v>2</v>
+      </c>
+      <c r="M14" s="80">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N14" s="80">
+        <v>300</v>
+      </c>
+      <c r="O14" s="91" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="84">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q14" s="84">
+        <f>P14*N14</f>
+        <v>0.38999999999999996</v>
+      </c>
+      <c r="R14" s="80"/>
+      <c r="S14" s="90"/>
+    </row>
+    <row r="15" spans="1:19" s="85" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="77"/>
+      <c r="B15" s="86">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="81" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="81" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="81">
+        <v>1</v>
+      </c>
+      <c r="M15" s="80">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N15" s="81">
+        <v>101</v>
+      </c>
+      <c r="O15" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="83">
+        <v>4.3240999999999996</v>
+      </c>
+      <c r="Q15" s="83">
+        <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
+        <v>436.73409999999996</v>
+      </c>
+      <c r="R15" s="81"/>
+      <c r="S15" s="92"/>
+    </row>
+    <row r="16" spans="1:19" s="85" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="77"/>
+      <c r="B16" s="86">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="79" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="81" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="81" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="81" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="81">
+        <v>1</v>
+      </c>
+      <c r="M16" s="80">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N16" s="81">
+        <v>100</v>
+      </c>
+      <c r="O16" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="83">
+        <v>0.64090000000000003</v>
+      </c>
+      <c r="Q16" s="83">
+        <f t="shared" si="4"/>
+        <v>64.09</v>
+      </c>
+      <c r="R16" s="81"/>
+      <c r="S16" s="92"/>
+    </row>
+    <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="48">
+        <f>SUM(Q10:Q16)</f>
+        <v>555.12279999999998</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
+    </row>
+    <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="49">
+        <f>Q17/100</f>
+        <v>5.5512280000000001</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="R17:S18"/>
+    <mergeCell ref="N18:P18"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O15" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="69"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="70"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="70"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="70"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="70"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="70"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="77"/>
+      <c r="B10" s="78">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="80" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="80" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="80" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="80" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="80" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="80">
+        <v>1</v>
+      </c>
+      <c r="M10" s="80">
+        <f>L10*500</f>
+        <v>500</v>
+      </c>
+      <c r="N10" s="81">
+        <v>600</v>
+      </c>
+      <c r="O10" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" s="83">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="Q10" s="84">
+        <f>P10*N10</f>
+        <v>3.1199999999999997</v>
+      </c>
+      <c r="R10" s="80"/>
+      <c r="S10" s="50"/>
+    </row>
+    <row r="11" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="77"/>
+      <c r="B11" s="86">
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="79" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="81" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="81" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="81" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="87" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="81" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="81" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="81" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="81">
+        <v>1</v>
+      </c>
+      <c r="M11" s="80">
+        <f t="shared" ref="M11:M16" si="1">L11*500</f>
+        <v>500</v>
+      </c>
+      <c r="N11" s="81">
+        <v>600</v>
+      </c>
+      <c r="O11" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="83">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q11" s="83">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>1.44</v>
+      </c>
+      <c r="R11" s="81"/>
+      <c r="S11" s="81"/>
+    </row>
+    <row r="12" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="77"/>
+      <c r="B12" s="78">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="87" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="87" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="87" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="87">
+        <v>1</v>
+      </c>
+      <c r="M12" s="80">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" s="89" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" s="89" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" s="87"/>
+      <c r="S12" s="90"/>
+    </row>
+    <row r="13" spans="1:19" s="85" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A13" s="77"/>
+      <c r="B13" s="86">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="79" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="81" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="81" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="81" t="s">
+        <v>71</v>
+      </c>
+      <c r="K13" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="81">
+        <v>1</v>
+      </c>
+      <c r="M13" s="80">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N13" s="81">
+        <v>502</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.47410000000000002</v>
+      </c>
+      <c r="Q13" s="83">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>237.9982</v>
+      </c>
+      <c r="R13" s="81"/>
+      <c r="S13" s="90"/>
+    </row>
+    <row r="14" spans="1:19" s="85" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="77"/>
+      <c r="B14" s="78">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="88" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="80" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="80" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="80" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="80" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="80" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="80" t="s">
+        <v>61</v>
+      </c>
+      <c r="K14" s="80" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="80">
+        <v>2</v>
+      </c>
+      <c r="M14" s="80">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N14" s="80">
+        <v>1100</v>
+      </c>
+      <c r="O14" s="91" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="84">
+        <v>1E-3</v>
+      </c>
+      <c r="Q14" s="84">
+        <f>P14*N14</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="R14" s="80"/>
+      <c r="S14" s="90"/>
+    </row>
+    <row r="15" spans="1:19" s="85" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="77"/>
+      <c r="B15" s="86">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="81" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="81" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="81">
+        <v>1</v>
+      </c>
+      <c r="M15" s="80">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N15" s="81">
+        <v>502</v>
+      </c>
+      <c r="O15" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="83">
+        <v>4.3240999999999996</v>
+      </c>
+      <c r="Q15" s="83">
+        <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
+        <v>2170.6981999999998</v>
+      </c>
+      <c r="R15" s="81"/>
+      <c r="S15" s="92"/>
+    </row>
+    <row r="16" spans="1:19" s="85" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="77"/>
+      <c r="B16" s="86">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="79" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="81" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="81" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="81" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="81" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="81">
+        <v>1</v>
+      </c>
+      <c r="M16" s="80">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N16" s="81">
+        <v>500</v>
+      </c>
+      <c r="O16" s="82" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="83">
+        <v>0.59709999999999996</v>
+      </c>
+      <c r="Q16" s="83">
+        <f t="shared" si="4"/>
+        <v>298.54999999999995</v>
+      </c>
+      <c r="R16" s="81"/>
+      <c r="S16" s="92"/>
+    </row>
+    <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="48">
+        <f>SUM(Q10:Q16)</f>
+        <v>2712.9063999999998</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
+    </row>
+    <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="49">
+        <f>Q17/500</f>
+        <v>5.4258128000000001</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="R17:S18"/>
+    <mergeCell ref="N18:P18"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O15" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId7"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="69"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="70"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="70"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="70"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="70"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="70"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="64"/>
+      <c r="B10" s="46">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="37">
+        <v>1</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="N10" s="51">
+        <v>1100</v>
+      </c>
+      <c r="O10" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P10" s="52">
+        <v>4.1000000000000003E-3</v>
+      </c>
+      <c r="Q10" s="38">
+        <f>P10*N10</f>
+        <v>4.5100000000000007</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="65"/>
+    </row>
+    <row r="11" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="64"/>
+      <c r="B11" s="47">
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="51" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="51" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="51">
+        <v>1</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M16" si="1">L11*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="N11" s="51">
+        <v>1100</v>
+      </c>
+      <c r="O11" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P11" s="52">
+        <v>1.8E-3</v>
+      </c>
+      <c r="Q11" s="52">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>1.98</v>
+      </c>
+      <c r="R11" s="51"/>
+      <c r="S11" s="51"/>
+    </row>
+    <row r="12" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="64"/>
+      <c r="B12" s="46">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="61">
+        <v>1</v>
+      </c>
+      <c r="M12" s="61">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="O12" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="P12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q12" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="R12" s="61"/>
+      <c r="S12" s="59"/>
+    </row>
+    <row r="13" spans="1:19" s="66" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="47">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="K13" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="51">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N13" s="51">
+        <v>1002</v>
+      </c>
+      <c r="O13" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P13" s="52">
+        <v>0.45190000000000002</v>
+      </c>
+      <c r="Q13" s="52">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>452.80380000000002</v>
+      </c>
+      <c r="R13" s="51"/>
+      <c r="S13" s="59"/>
+    </row>
+    <row r="14" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="64"/>
+      <c r="B14" s="46">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="37">
+        <v>2</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="N14" s="37">
+        <v>2100</v>
+      </c>
+      <c r="O14" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="P14" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q14" s="38">
+        <f>P14*N14</f>
+        <v>2.1</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="59"/>
+    </row>
+    <row r="15" spans="1:19" s="66" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="64"/>
+      <c r="B15" s="47">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L15" s="51">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N15" s="51">
+        <v>1002</v>
+      </c>
+      <c r="O15" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="52">
+        <v>4.3240999999999996</v>
+      </c>
+      <c r="Q15" s="52">
+        <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
+        <v>4332.7482</v>
+      </c>
+      <c r="R15" s="51"/>
+      <c r="S15" s="39"/>
+    </row>
+    <row r="16" spans="1:19" s="66" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="64"/>
+      <c r="B16" s="47">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="54" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="51">
+        <v>1</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N16" s="51">
+        <v>1000</v>
+      </c>
+      <c r="O16" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="P16" s="52">
+        <v>0.57750000000000001</v>
+      </c>
+      <c r="Q16" s="52">
+        <f t="shared" si="4"/>
+        <v>577.5</v>
+      </c>
+      <c r="R16" s="51"/>
+      <c r="S16" s="39"/>
+    </row>
+    <row r="17" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="48">
+        <f>SUM(Q10:Q16)</f>
+        <v>5371.6419999999998</v>
+      </c>
+      <c r="R17" s="71"/>
+      <c r="S17" s="72"/>
+    </row>
+    <row r="18" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="49">
+        <f>Q17/1000</f>
+        <v>5.3716419999999996</v>
+      </c>
+      <c r="R18" s="73"/>
+      <c r="S18" s="74"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="R17:S18"/>
+    <mergeCell ref="N18:P18"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O15" r:id="rId3"/>
+    <hyperlink ref="O14" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O13" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>